<commit_message>
Add PL-600 study artifacts and completed workbook
</commit_message>
<xml_diff>
--- a/Allfiles/Project Workbook PL-600 Applied Exercise.xlsx
+++ b/Allfiles/Project Workbook PL-600 Applied Exercise.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ctcvso\MSFT Applied Exercises\Current\PL600 Power Platform Solution Architect\capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cba37b90ae6b55a9/Desktop/pl-600/NetcomExcersise/NetCom/PL-600-Microsoft-Power-Platform-Solution-Architect/Allfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E7D880-0333-455C-AFE5-1ADBD4C9B1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{13E7D880-0333-455C-AFE5-1ADBD4C9B1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49DC13BF-42A6-482D-A448-9C3EEAED65C8}"/>
   <bookViews>
-    <workbookView xWindow="-30310" yWindow="1900" windowWidth="27380" windowHeight="15370" firstSheet="1" activeTab="6" xr2:uid="{A7FE3A90-ABDE-4482-A392-34584F34D645}"/>
+    <workbookView xWindow="-35490" yWindow="5535" windowWidth="28800" windowHeight="15345" firstSheet="1" activeTab="6" xr2:uid="{A7FE3A90-ABDE-4482-A392-34584F34D645}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Discovery" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="143">
   <si>
     <t>Description</t>
   </si>
@@ -241,12 +241,6 @@
     <t>Your development team has implemented a Power Automate flow that sends the resolution back to the originating system. During testing, the test team has identified if the originating system is down the resolution doesn't get recorded because the cloud flow fails. How would you advise your development team to improve the reliability of the integration?</t>
   </si>
   <si>
-    <t>Insert your high level architecture diagram here</t>
-  </si>
-  <si>
-    <t>Insert your high level data model diagram here</t>
-  </si>
-  <si>
     <t>Question</t>
   </si>
   <si>
@@ -307,7 +301,199 @@
     <t>Additional considerations</t>
   </si>
   <si>
-    <t>Insert your high leve ALM plan here</t>
+    <t>Fabrikam Home Systems (fictitious)</t>
+  </si>
+  <si>
+    <t>Seattle, Washington, USA</t>
+  </si>
+  <si>
+    <t>United Kingdom, India, Germany, Canada</t>
+  </si>
+  <si>
+    <t>Ava Patel (CEO), Marcus Lee (COO), Elena Rossi (CIO)</t>
+  </si>
+  <si>
+    <t>Microsoft Azure (primary), limited AWS for legacy workloads</t>
+  </si>
+  <si>
+    <t>Power Platform first strategy, API-first integrations, Dataverse-centric architecture</t>
+  </si>
+  <si>
+    <t>Smart bed manufacturing, support subscriptions, field maintenance services</t>
+  </si>
+  <si>
+    <t>Pain points: high cancellation volume, slow case triage, fragmented customer history, weak proactive retention analytics</t>
+  </si>
+  <si>
+    <t>High-level architecture (study view):
+Channels: Phone, Email, Web Chat/Portal, Social -&gt; Omnichannel + Customer Service
+Core: Dataverse + Dynamics 365 Customer Service (cases, SLAs, queues, knowledge)
+Retention: Sales Enterprise for upsell/cross-sell + discount approval process
+Automation: Power Automate cloud flows, approval flows, scheduled archival/deletion
+Integration: API Mgmt + custom connectors + Service Bus for reliable outbound callbacks
+Insights: Power BI real-time dashboards for executives and managers
+Identity/Security: Entra ID groups, Business Units, Teams, DLP policies</t>
+  </si>
+  <si>
+    <t>Use Dataverse + Service Bus + API Management for resilient integration patterns</t>
+  </si>
+  <si>
+    <t>Yes - Routing, approvals, notifications, integrations</t>
+  </si>
+  <si>
+    <t>Yes - Website bot for status and FAQ</t>
+  </si>
+  <si>
+    <t>Yes - Executive and operations dashboards</t>
+  </si>
+  <si>
+    <t>Yes - Customer portal for status and self-service</t>
+  </si>
+  <si>
+    <t>Yes - Onsite dispatch when needed</t>
+  </si>
+  <si>
+    <t>Yes - Manager KPIs and support analytics</t>
+  </si>
+  <si>
+    <t>Yes - Case/queue/SLA/knowledge/omnichannel</t>
+  </si>
+  <si>
+    <t>Optional - Forecasting retention outcomes</t>
+  </si>
+  <si>
+    <t>Yes - Retention offers and contract upgrades</t>
+  </si>
+  <si>
+    <t>Yes - Agent assist app + supervisor console</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Configure</t>
+  </si>
+  <si>
+    <t>Power BI DirectQuery/near real-time tiles for success/failure, SLA and churn KPIs.</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Performance design: regional environments, optimized forms, async operations, indexing.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>OOB</t>
+  </si>
+  <si>
+    <t>Use created/resolved dates and calculated columns for aging metrics.</t>
+  </si>
+  <si>
+    <t>Scheduled and event-based reminders for overdue follow-ups.</t>
+  </si>
+  <si>
+    <t>Sentiment detection + keyword rules to notify manager and copy communications.</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Portal page for authenticated users to view request progress and milestones.</t>
+  </si>
+  <si>
+    <t>SLA KPI instances and escalation dashboards for managers.</t>
+  </si>
+  <si>
+    <t>Email template + flow on resolution status change.</t>
+  </si>
+  <si>
+    <t>Guided process to create discounted offer and convert to new service agreement.</t>
+  </si>
+  <si>
+    <t>My Open Requests view + timeline + follow-up date indicators and reminders.</t>
+  </si>
+  <si>
+    <t>Near real-time ingestion via Event Hub/Service Bus + Power Automate/Azure Function to Dataverse.</t>
+  </si>
+  <si>
+    <t>Model offers table and role-based views with recommendation rules.</t>
+  </si>
+  <si>
+    <t>Use Power Pages + Copilot Studio bot + Dataverse virtual table/API for live status.</t>
+  </si>
+  <si>
+    <t>Use queue views and work item assignment in Customer Service workspace.</t>
+  </si>
+  <si>
+    <t>Use unified routing rules + queue assignment based on skill and open workload.</t>
+  </si>
+  <si>
+    <t>High-level data model (study view):
+Account 1-* Contact
+Account 1-* Service Agreement
+Account 1-* Complaint/Cancel Request
+Complaint *-1 Originating System
+Complaint 1-* Activity (calls/emails/tasks)
+Complaint 1-* Offer
+Offer *-1 Manager Approver (User)
+Complaint 1-* SLA KPI Instance
+Complaint 1-* Integration Event (outbound status/retry)
+Reference tables: Reason, Channel, Priority, Sentiment, Resolution Type</t>
+  </si>
+  <si>
+    <t>User groups: Retention agents, Retention managers, Executives, Customers, Integration support/admins.</t>
+  </si>
+  <si>
+    <t>Model-driven app (Retention Hub) for agents/managers; Power Pages portal for customers; optional canvas supervisor board; Copilot Studio bot for website chat.</t>
+  </si>
+  <si>
+    <t>PCF: SLA countdown timer, sentiment indicator control, discount approval badge, timeline summarizer, retry status control for integrations.</t>
+  </si>
+  <si>
+    <t>Automate routing, reminders, customer notifications, approval workflows, outbound callbacks, nightly archiving/deletion, KPI refresh orchestration.</t>
+  </si>
+  <si>
+    <t>Publish a reliable outbound event from Dataverse to Service Bus, process via cloud flow/Azure Function with retry, dead-letter queue, and reconciliation job.</t>
+  </si>
+  <si>
+    <t>Prefer cloud flow + queue-based integration over plug-in. Trigger on resolved complaint, transform payload, send via webhook/API, and log delivery result.</t>
+  </si>
+  <si>
+    <t>Scheduled cloud flow runs daily: find resolved complaints older than 28 days, archive required fields to lake/storage, then delete/anonymize records in Dataverse.</t>
+  </si>
+  <si>
+    <t>Approval flow triggered when discount &gt; 50%; route to retention manager, lock status pending approval, auto-notify agent/customer, and audit all decisions.</t>
+  </si>
+  <si>
+    <t>Implement resilient pattern: asynchronous queue, retry with exponential backoff, idempotency key, dead-letter queue, alerting, and replay flow for failures.</t>
+  </si>
+  <si>
+    <t>Roles: Retention Agent, Retention Manager, Executive Read-Only, Integration Service Role, Portal Customer, System Admin. Restrict table/field access by least privilege.</t>
+  </si>
+  <si>
+    <t>Business Units: Global Root; Americas Retention; EMEA Retention; APAC Retention; Shared Services. Managers get BU/parent-child visibility; agents mostly user/team scope.</t>
+  </si>
+  <si>
+    <t>Teams: Small Deals Team (shared visibility), Enterprise Deal Pods (access teams per case), Escalation Team, Integration Ops Team.</t>
+  </si>
+  <si>
+    <t>Entra ID Groups: RetentionAgents, RetentionManagers, Executives, IntegrationAdmins, PortalSupport. Use group teams for automated role assignment and app access.</t>
+  </si>
+  <si>
+    <t>High-level ALM plan:
+1) Environments: Dev -&gt; Test/UAT -&gt; Prod (plus training sandbox).
+2) Solutions: Core Data, Apps, Automation, Integrations, Reporting split into managed layers.
+3) Source control: unpacked solutions in Git with branch policies + PR reviews.
+4) Pipelines: build/validate/export/import with connection references and environment variables.
+5) Quality gates: solution checker, automated tests, performance smoke tests, security review.
+6) Release strategy: weekly minor releases, monthly feature releases, rollback package retained.
+7) Governance: DLP policies, naming standards, telemetry, and operational runbooks.</t>
   </si>
 </sst>
 </file>
@@ -403,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -427,6 +613,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,9 +632,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -485,7 +672,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -591,7 +778,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -733,7 +920,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -742,13 +929,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{143EFBDA-0A2F-4F44-AA9B-25D61515829C}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" customWidth="1"/>
+    <col min="1" max="1" width="44.85546875" customWidth="1"/>
     <col min="2" max="2" width="92" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>50</v>
       </c>
@@ -756,49 +943,76 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="36.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="36.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="9">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="38.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="37" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>85</v>
+      <c r="B11" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -810,14 +1024,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E27BCEE7-F14E-46D1-80D5-EEBCCD0F485E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="79.81640625" customWidth="1"/>
+    <col min="1" max="1" width="79.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
-        <v>66</v>
+    <row r="1" spans="1:1" s="5" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -828,163 +1042,196 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F14C17BB-8A79-4424-BD4B-A71907C20423}">
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.54296875" customWidth="1"/>
-    <col min="2" max="2" width="34.81640625" customWidth="1"/>
+    <col min="1" max="1" width="44.5703125" customWidth="1"/>
+    <col min="2" max="2" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>87</v>
+        <v>85</v>
+      </c>
+      <c r="B31" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -995,17 +1242,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E84F61-9550-43C2-997B-E7403D84F0A0}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="57.453125" customWidth="1"/>
-    <col min="3" max="3" width="18.81640625" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" customWidth="1"/>
-    <col min="5" max="5" width="29.453125" customWidth="1"/>
-    <col min="6" max="6" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="57.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>5</v>
       </c>
@@ -1025,7 +1272,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="5" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" s="5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
@@ -1042,124 +1289,304 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>8</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>9</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>10</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E10" t="s">
+        <v>113</v>
+      </c>
+      <c r="F10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>11</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>12</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" t="s">
+        <v>117</v>
+      </c>
+      <c r="F12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>13</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>14</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>15</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>17</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>18</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" t="s">
+        <v>108</v>
+      </c>
+      <c r="F17" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1171,14 +1598,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C0F67D-032F-41B8-998C-86CA2E86B6C0}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.81640625" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>67</v>
+    <row r="1" spans="1:1" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1189,13 +1616,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14AA0956-51E3-4088-B675-3384AECDD7E4}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.453125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="86.453125" customWidth="1"/>
+    <col min="1" max="1" width="55.42578125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="86.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>53</v>
       </c>
@@ -1203,29 +1630,44 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="69" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="65.150000000000006" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1237,13 +1679,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F3EEEA2-6773-4CE0-ADFF-280F7CC91CAD}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="73.1796875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="92.7265625" customWidth="1"/>
+    <col min="1" max="1" width="73.140625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="92.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>59</v>
       </c>
@@ -1251,30 +1693,42 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="66.650000000000006" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="7" spans="1:2" ht="63.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:2" ht="63.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="76" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="75.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>65</v>
+      </c>
+      <c r="B9" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1285,43 +1739,55 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE3C611-38C7-4EE1-8F61-078D836311E9}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="75.453125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="75.54296875" customWidth="1"/>
+    <col min="1" max="1" width="75.42578125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="75.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:2" ht="44.15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:2" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:2" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:2" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="49" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="B10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="48.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1330,14 +1796,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397C6D9D-BC0B-4AE6-A231-75899A24C784}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="54.81640625" customWidth="1"/>
+    <col min="1" max="1" width="54.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>88</v>
+    <row r="1" spans="1:1" ht="219.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1346,6 +1812,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="a27ad7fd-960b-41e4-8b5b-7279e52d6f14" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7cab2185-db21-48eb-be1e-592331867472">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100448DCFA98101424CAAC1CCC7B479C823" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ce40a7b3e3337de2864492f4180f194f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7cab2185-db21-48eb-be1e-592331867472" xmlns:ns3="a27ad7fd-960b-41e4-8b5b-7279e52d6f14" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="109ae85b6bb81c9d3b2f22784c06469d" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1579,38 +2067,44 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="a27ad7fd-960b-41e4-8b5b-7279e52d6f14" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7cab2185-db21-48eb-be1e-592331867472">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E9A1888-2A1D-4464-A773-357CAC01C36C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E7831EA-5C0B-42F7-9E64-4C69715018BC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="a27ad7fd-960b-41e4-8b5b-7279e52d6f14"/>
+    <ds:schemaRef ds:uri="7cab2185-db21-48eb-be1e-592331867472"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E55B014-9601-47A9-A1BB-8E52BFCA08F0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E55B014-9601-47A9-A1BB-8E52BFCA08F0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E7831EA-5C0B-42F7-9E64-4C69715018BC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E9A1888-2A1D-4464-A773-357CAC01C36C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="7cab2185-db21-48eb-be1e-592331867472"/>
+    <ds:schemaRef ds:uri="a27ad7fd-960b-41e4-8b5b-7279e52d6f14"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>